<commit_message>
updated home_visit.py not loss when network gone.
</commit_message>
<xml_diff>
--- a/movement.xlsx
+++ b/movement.xlsx
@@ -8,17 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91730\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800D6E04-263C-4EE7-A30A-1DEB9D4537C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98991522-EAE9-44AA-B674-E91E32F3C609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1037,7 +1046,7 @@
         <v>42</v>
       </c>
       <c r="C2" s="2">
-        <v>200</v>
+        <v>369</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
@@ -1141,7 +1150,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="2">
-        <v>200</v>
+        <v>358</v>
       </c>
       <c r="D3" s="10">
         <v>83</v>
@@ -1245,7 +1254,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="2">
-        <v>200</v>
+        <v>348</v>
       </c>
       <c r="D4" s="10">
         <v>164</v>
@@ -1349,7 +1358,7 @@
         <v>43</v>
       </c>
       <c r="C5" s="2">
-        <v>200</v>
+        <v>266</v>
       </c>
       <c r="D5" s="10">
         <v>247</v>
@@ -1453,7 +1462,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="2">
-        <v>200</v>
+        <v>281</v>
       </c>
       <c r="D6" s="10">
         <v>317</v>
@@ -1557,7 +1566,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="2">
-        <v>200</v>
+        <v>336</v>
       </c>
       <c r="D7" s="10">
         <v>376</v>
@@ -1661,7 +1670,7 @@
         <v>44</v>
       </c>
       <c r="C8" s="2">
-        <v>200</v>
+        <v>443</v>
       </c>
       <c r="D8" s="10">
         <v>434</v>
@@ -1765,7 +1774,7 @@
         <v>45</v>
       </c>
       <c r="C9" s="2">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="D9" s="10">
         <v>510</v>
@@ -1869,7 +1878,7 @@
         <v>46</v>
       </c>
       <c r="C10" s="2">
-        <v>200</v>
+        <v>276</v>
       </c>
       <c r="D10" s="10">
         <v>573</v>
@@ -1973,7 +1982,7 @@
         <v>47</v>
       </c>
       <c r="C11" s="19">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="D11" s="13">
         <v>628</v>

</xml_diff>